<commit_message>
Added default option for Environment Class constructor
</commit_message>
<xml_diff>
--- a/Environment/WindParameters.xlsx
+++ b/Environment/WindParameters.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahrid\OneDrive\Desktop\GeorgiaTech\Clubs\GNC\Github2\GNCSIM\WindMonteCarlo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahrid\OneDrive\Desktop\GT Clubs\GNC\GNCSIM GITHUB\GNCSIM\Environment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4115CA8-77CE-46CB-8FC8-BB902707DF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABB992B-B6DD-4BEC-BD8E-D93AE66D6A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6510" yWindow="4515" windowWidth="29010" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -394,19 +394,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" customWidth="1"/>
-    <col min="2" max="2" width="19.5546875" customWidth="1"/>
-    <col min="3" max="3" width="23.5546875" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" customWidth="1"/>
-    <col min="5" max="5" width="21.44140625" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" customWidth="1"/>
-    <col min="8" max="8" width="17.5546875" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -432,7 +432,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -458,7 +458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -484,7 +484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -510,7 +510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>

</xml_diff>